<commit_message>
fix: Updated timesheet formatting, visual changes
</commit_message>
<xml_diff>
--- a/public/timesheet.xlsx
+++ b/public/timesheet.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t xml:space="preserve">WhereToNext/MED</t>
   </si>
@@ -80,6 +80,9 @@
   </si>
   <si>
     <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task(s)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL  </t>
@@ -89,13 +92,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mmmm\ d&quot;, &quot;yyyy"/>
     <numFmt numFmtId="166" formatCode="mmm\ d&quot;, &quot;yyyy"/>
-    <numFmt numFmtId="167" formatCode="hh:mm:ss\ AM/PM"/>
-    <numFmt numFmtId="168" formatCode="h:mm:ss"/>
-    <numFmt numFmtId="169" formatCode="h:mm"/>
+    <numFmt numFmtId="167" formatCode="hh:mm\ AM/PM"/>
+    <numFmt numFmtId="168" formatCode="h:mm\ AM/PM"/>
+    <numFmt numFmtId="169" formatCode="h:mm:ss"/>
+    <numFmt numFmtId="170" formatCode="h:mm"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -242,7 +246,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -335,11 +339,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="170" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -426,9 +434,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1449720</xdr:colOff>
+      <xdr:colOff>1449000</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>37440</xdr:rowOff>
+      <xdr:rowOff>36720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -442,7 +450,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="81360" y="0"/>
-          <a:ext cx="1368360" cy="1368360"/>
+          <a:ext cx="1367640" cy="1367640"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -574,7 +582,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="22.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="15.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="29.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="46" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -733,7 +741,9 @@
       <c r="G10" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="H10" s="6"/>
+      <c r="H10" s="18" t="s">
+        <v>20</v>
+      </c>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
     </row>
@@ -744,13 +754,13 @@
       <c r="B11" s="20"/>
       <c r="C11" s="21"/>
       <c r="D11" s="21"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="22" t="n">
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="23" t="n">
         <f aca="false">IF($D11&lt;$C11,$D11+12-$C11,$D11-$C11)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="6"/>
+      <c r="H11" s="19"/>
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
     </row>
@@ -760,14 +770,14 @@
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
-      <c r="F12" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="24" t="n">
+      <c r="F12" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="25" t="n">
         <f aca="false">SUM($G$11:$G11)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="6"/>
+      <c r="H12" s="19"/>
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
     </row>

</xml_diff>